<commit_message>
pushing after testing completed
</commit_message>
<xml_diff>
--- a/results/findings.xlsx
+++ b/results/findings.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IBA\Thesis\Implementation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IBA\Thesis\Implementation\Advancements-in-Ensemble-Learning\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3DD01E2-8D94-49D1-A443-0A172DAAF80C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1186284-362A-4A4C-979B-A63E3E79B248}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{C2C4D7A9-A02F-4765-9375-2B79B66B31F3}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="82">
   <si>
     <t>Datasets</t>
   </si>
@@ -134,6 +134,144 @@
   </si>
   <si>
     <t>XGBoost</t>
+  </si>
+  <si>
+    <t>K=power(n,1/3), no homogenous clusters</t>
+  </si>
+  <si>
+    <t>1h 10m</t>
+  </si>
+  <si>
+    <t>duration</t>
+  </si>
+  <si>
+    <t>Fuzzy Kmean</t>
+  </si>
+  <si>
+    <t>1h 20m</t>
+  </si>
+  <si>
+    <t>Adding diversity to PSO 2</t>
+  </si>
+  <si>
+    <t>1h 23m</t>
+  </si>
+  <si>
+    <t>1h 15m</t>
+  </si>
+  <si>
+    <t>Hierarical Clustering</t>
+  </si>
+  <si>
+    <t>Hierarical Clustering (avg 10)</t>
+  </si>
+  <si>
+    <t>Kmean using Elbow Methos</t>
+  </si>
+  <si>
+    <t>57s</t>
+  </si>
+  <si>
+    <t>32s</t>
+  </si>
+  <si>
+    <t>26s</t>
+  </si>
+  <si>
+    <t>31s</t>
+  </si>
+  <si>
+    <t>16s</t>
+  </si>
+  <si>
+    <t>45s</t>
+  </si>
+  <si>
+    <t>1m 3s</t>
+  </si>
+  <si>
+    <t>20s</t>
+  </si>
+  <si>
+    <t>19s</t>
+  </si>
+  <si>
+    <t>1m 5s</t>
+  </si>
+  <si>
+    <t>38s</t>
+  </si>
+  <si>
+    <t>37s</t>
+  </si>
+  <si>
+    <t>41s</t>
+  </si>
+  <si>
+    <t>21s</t>
+  </si>
+  <si>
+    <t>1m 2s</t>
+  </si>
+  <si>
+    <t>1m 20s</t>
+  </si>
+  <si>
+    <t>37m 17s</t>
+  </si>
+  <si>
+    <t>25s</t>
+  </si>
+  <si>
+    <t>23s</t>
+  </si>
+  <si>
+    <t>replacing PSO2 with SHAP</t>
+  </si>
+  <si>
+    <t>27s</t>
+  </si>
+  <si>
+    <t>9s</t>
+  </si>
+  <si>
+    <t>12s</t>
+  </si>
+  <si>
+    <t>11s</t>
+  </si>
+  <si>
+    <t>40m 26s</t>
+  </si>
+  <si>
+    <t>excluding PSO1</t>
+  </si>
+  <si>
+    <t>36s</t>
+  </si>
+  <si>
+    <t>34s</t>
+  </si>
+  <si>
+    <t>50s</t>
+  </si>
+  <si>
+    <t>18s</t>
+  </si>
+  <si>
+    <t>39m 39s</t>
+  </si>
+  <si>
+    <t>credit-card-default</t>
+  </si>
+  <si>
+    <t>46m 54s</t>
+  </si>
+  <si>
+    <t>bank-marketing</t>
+  </si>
+  <si>
+    <t>33m 23s</t>
   </si>
 </sst>
 </file>
@@ -272,15 +410,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
@@ -288,7 +426,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
@@ -296,10 +433,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
@@ -852,25 +985,31 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81B84C67-EC3E-43AB-8AFA-1799144B48B6}">
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:AQ14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="8.88671875" style="15"/>
-    <col min="3" max="3" width="8.88671875" style="16"/>
-    <col min="4" max="4" width="8.88671875" style="17"/>
-    <col min="5" max="5" width="8.88671875" style="16"/>
-    <col min="6" max="6" width="8.88671875" style="17"/>
-    <col min="7" max="7" width="8.88671875" style="16"/>
-    <col min="8" max="8" width="8.88671875" style="15"/>
-    <col min="9" max="9" width="8.88671875" style="16"/>
-    <col min="10" max="10" width="8.88671875" style="15"/>
-    <col min="11" max="11" width="8.88671875" style="16"/>
-    <col min="13" max="13" width="8.88671875" style="16"/>
-    <col min="15" max="15" width="8.88671875" style="16"/>
-    <col min="16" max="16" width="8.88671875" style="28"/>
+    <col min="3" max="3" width="8.88671875" style="15"/>
+    <col min="4" max="4" width="8.88671875" style="16"/>
+    <col min="5" max="5" width="8.88671875" style="15"/>
+    <col min="6" max="6" width="8.88671875" style="16"/>
+    <col min="7" max="7" width="8.88671875" style="15"/>
+    <col min="9" max="9" width="8.88671875" style="15"/>
+    <col min="11" max="11" width="8.88671875" style="15"/>
+    <col min="13" max="13" width="8.88671875" style="15"/>
+    <col min="15" max="15" width="8.88671875" style="15"/>
+    <col min="16" max="16" width="8.88671875" style="23"/>
+    <col min="19" max="19" width="8.88671875" style="15"/>
+    <col min="22" max="22" width="8.88671875" style="15"/>
+    <col min="25" max="25" width="8.88671875" style="15"/>
+    <col min="28" max="28" width="8.88671875" style="15"/>
+    <col min="31" max="31" width="8.88671875" style="15"/>
+    <col min="34" max="34" width="8.88671875" style="15"/>
+    <col min="37" max="37" width="8.88671875" style="15"/>
+    <col min="40" max="40" width="8.88671875" style="15"/>
+    <col min="43" max="43" width="8.88671875" style="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:43" s="7" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -880,11 +1019,11 @@
       <c r="C1" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="17" t="s">
         <v>10</v>
       </c>
       <c r="E1" s="8"/>
-      <c r="F1" s="18" t="s">
+      <c r="F1" s="17" t="s">
         <v>25</v>
       </c>
       <c r="G1" s="8"/>
@@ -904,441 +1043,1039 @@
         <v>29</v>
       </c>
       <c r="O1" s="8"/>
-      <c r="P1" s="27" t="s">
+      <c r="P1" s="22" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" s="19" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="C2" s="20"/>
-      <c r="D2" s="22" t="s">
+      <c r="Q1" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="S1" s="8"/>
+      <c r="T1" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="V1" s="8"/>
+      <c r="W1" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y1" s="8"/>
+      <c r="Z1" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="AB1" s="8"/>
+      <c r="AC1" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="AE1" s="8"/>
+      <c r="AF1" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="AH1" s="8"/>
+      <c r="AI1" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="AK1" s="8"/>
+      <c r="AL1" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN1" s="8"/>
+      <c r="AO1" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="AQ1" s="8"/>
+    </row>
+    <row r="2" spans="1:43" s="18" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C2" s="19"/>
+      <c r="D2" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="E2" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="21"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="24" t="s">
+      <c r="F2" s="20"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="I2" s="20" t="s">
+      <c r="I2" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="J2" s="23" t="s">
+      <c r="J2" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="K2" s="20" t="s">
+      <c r="K2" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="L2" s="23" t="s">
+      <c r="L2" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="20" t="s">
+      <c r="M2" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="N2" s="23" t="s">
+      <c r="N2" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="O2" s="20" t="s">
+      <c r="O2" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="P2" s="22" t="s">
+      <c r="P2" s="21" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A3" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="15" t="s">
+      <c r="Q2" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="R2" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="S2" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="T2" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="U2" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="V2" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="W2" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="X2" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y2" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="Z2" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="AA2" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="AB2" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="AC2" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD2" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="AE2" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="AF2" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="AG2" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="AH2" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="AI2" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="AJ2" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="AK2" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="AL2" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="AM2" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="AN2" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="AO2" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="AP2" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="AQ2" s="21" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="16">
+      <c r="C3" s="15">
         <v>2</v>
       </c>
-      <c r="D3" s="17">
+      <c r="D3" s="16">
         <v>0.96399999999999997</v>
       </c>
-      <c r="E3" s="16">
+      <c r="E3" s="15">
         <v>2.48E-3</v>
       </c>
-      <c r="H3" s="15">
+      <c r="H3">
         <v>0.9708</v>
       </c>
-      <c r="I3" s="16">
+      <c r="I3" s="15">
         <v>0.9708</v>
       </c>
-      <c r="J3" s="15">
+      <c r="J3">
         <v>0.97809999999999997</v>
       </c>
-      <c r="K3" s="16">
+      <c r="K3" s="15">
         <v>0.9708</v>
       </c>
-      <c r="L3" s="25">
+      <c r="L3">
         <v>0.9708</v>
       </c>
-      <c r="M3" s="26">
+      <c r="M3" s="15">
         <v>0.97809999999999997</v>
       </c>
-      <c r="N3" s="25">
+      <c r="N3">
         <v>0.9708</v>
       </c>
-      <c r="O3" s="16">
+      <c r="O3" s="15">
         <v>0.96350000000000002</v>
       </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A4" s="15" t="s">
+      <c r="AC3">
+        <v>0.92330000000000001</v>
+      </c>
+      <c r="AD3">
+        <v>0.90139999999999998</v>
+      </c>
+      <c r="AF3">
+        <v>0.42335766423357601</v>
+      </c>
+      <c r="AG3">
+        <v>0.58394160583941601</v>
+      </c>
+      <c r="AH3" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="AI3">
+        <v>0.42335766423357601</v>
+      </c>
+      <c r="AJ3">
+        <v>0.42335766423357601</v>
+      </c>
+      <c r="AK3" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="AL3">
+        <v>0.94890510948905105</v>
+      </c>
+      <c r="AM3">
+        <v>0.95620437956204296</v>
+      </c>
+      <c r="AN3" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO3">
+        <v>0.95620437956204296</v>
+      </c>
+      <c r="AP3">
+        <v>0.96350364963503599</v>
+      </c>
+      <c r="AQ3" s="15" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="16">
+      <c r="C4" s="15">
         <v>8</v>
       </c>
-      <c r="D4" s="17">
+      <c r="D4" s="16">
         <v>0.95099999999999996</v>
       </c>
-      <c r="E4" s="16">
+      <c r="E4" s="15">
         <v>3.2000000000000003E-4</v>
       </c>
-      <c r="H4" s="15">
+      <c r="H4">
         <v>0.98519999999999996</v>
       </c>
-      <c r="I4" s="16">
+      <c r="I4" s="15">
         <v>0.98519999999999996</v>
       </c>
-      <c r="J4" s="15">
+      <c r="J4">
         <v>0.98519999999999996</v>
       </c>
-      <c r="K4" s="16">
+      <c r="K4" s="15">
         <v>0.9264</v>
       </c>
-      <c r="L4" s="15">
+      <c r="L4">
         <v>0.98519999999999996</v>
       </c>
-      <c r="M4" s="16">
+      <c r="M4" s="15">
         <v>0.98519999999999996</v>
       </c>
-      <c r="N4" s="15">
+      <c r="N4">
         <v>0.98519999999999996</v>
       </c>
-      <c r="O4" s="16">
+      <c r="O4" s="15">
         <v>0.98519999999999996</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A5" s="15" t="s">
+      <c r="AC4">
+        <v>0.79410000000000003</v>
+      </c>
+      <c r="AD4">
+        <v>0.8014</v>
+      </c>
+      <c r="AF4">
+        <v>0.32352941176470501</v>
+      </c>
+      <c r="AG4">
+        <v>0.441176470588235</v>
+      </c>
+      <c r="AH4" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI4">
+        <v>0.47058823529411697</v>
+      </c>
+      <c r="AJ4">
+        <v>0.47058823529411697</v>
+      </c>
+      <c r="AK4" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="AL4">
+        <v>0.94117647058823495</v>
+      </c>
+      <c r="AM4">
+        <v>0.64705882352941102</v>
+      </c>
+      <c r="AN4" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="AO4">
+        <v>0.98529411764705799</v>
+      </c>
+      <c r="AP4">
+        <v>0.97058823529411697</v>
+      </c>
+      <c r="AQ4" s="15" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="16">
+      <c r="C5" s="15">
         <v>2</v>
       </c>
-      <c r="D5" s="17">
+      <c r="D5" s="16">
         <v>0.748</v>
       </c>
-      <c r="E5" s="16">
+      <c r="E5" s="15">
         <v>2.0200000000000001E-3</v>
       </c>
-      <c r="H5" s="15">
+      <c r="H5">
         <v>0.78680000000000005</v>
       </c>
-      <c r="I5" s="16">
+      <c r="I5" s="15">
         <v>0.78680000000000005</v>
       </c>
-      <c r="J5" s="15">
+      <c r="J5">
         <v>0.77039999999999997</v>
       </c>
-      <c r="K5" s="16">
+      <c r="K5" s="15">
         <v>0.80320000000000003</v>
       </c>
-      <c r="L5" s="25">
+      <c r="L5">
         <v>0.77039999999999997</v>
       </c>
-      <c r="M5" s="26">
+      <c r="M5" s="15">
         <v>0.77039999999999997</v>
       </c>
-      <c r="N5" s="25">
+      <c r="N5">
         <v>0.78680000000000005</v>
       </c>
-      <c r="O5" s="26">
+      <c r="O5" s="15">
         <v>0.77039999999999997</v>
       </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A6" s="15" t="s">
+      <c r="AC5">
+        <v>0.73770000000000002</v>
+      </c>
+      <c r="AD5">
+        <v>0.74590000000000001</v>
+      </c>
+      <c r="AF5">
+        <v>0.68852459016393397</v>
+      </c>
+      <c r="AG5">
+        <v>0.67213114754098302</v>
+      </c>
+      <c r="AH5" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="AI5">
+        <v>0.70491803278688503</v>
+      </c>
+      <c r="AJ5">
+        <v>0.70491803278688503</v>
+      </c>
+      <c r="AK5" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="AL5">
+        <v>0.72131147540983598</v>
+      </c>
+      <c r="AM5">
+        <v>0.75409836065573699</v>
+      </c>
+      <c r="AN5" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="AO5">
+        <v>0.73770491803278604</v>
+      </c>
+      <c r="AP5">
+        <v>0.73770491803278604</v>
+      </c>
+      <c r="AQ5" s="15" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="16">
+      <c r="C6" s="15">
         <v>2</v>
       </c>
-      <c r="D6" s="17">
+      <c r="D6" s="16">
         <v>0.91700000000000004</v>
       </c>
-      <c r="E6" s="16">
+      <c r="E6" s="15">
         <v>3.2799999999999999E-3</v>
       </c>
-      <c r="H6" s="15">
+      <c r="H6">
         <v>0.81689999999999996</v>
       </c>
-      <c r="I6" s="16">
+      <c r="I6" s="15">
         <v>0.87319999999999998</v>
       </c>
-      <c r="J6" s="25">
+      <c r="J6">
         <v>0.91539999999999999</v>
       </c>
-      <c r="K6" s="26">
+      <c r="K6" s="15">
         <v>0.91539999999999999</v>
       </c>
-      <c r="L6" s="25">
+      <c r="L6">
         <v>0.94359999999999999</v>
       </c>
-      <c r="M6" s="26">
+      <c r="M6" s="15">
         <v>0.90139999999999998</v>
       </c>
-      <c r="N6" s="25">
+      <c r="N6">
         <v>0.91539999999999999</v>
       </c>
-      <c r="O6" s="16">
+      <c r="O6" s="15">
         <v>0.92949999999999999</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A7" s="15" t="s">
+      <c r="AC6">
+        <v>0.87319999999999998</v>
+      </c>
+      <c r="AD6">
+        <v>0.86609999999999998</v>
+      </c>
+      <c r="AF6">
+        <v>0.60563380281690105</v>
+      </c>
+      <c r="AG6">
+        <v>0.59154929577464699</v>
+      </c>
+      <c r="AH6" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="AI6">
+        <v>0.63380281690140805</v>
+      </c>
+      <c r="AJ6">
+        <v>0.60563380281690105</v>
+      </c>
+      <c r="AK6" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="AL6">
+        <v>0.91549295774647799</v>
+      </c>
+      <c r="AM6">
+        <v>0.90140845070422504</v>
+      </c>
+      <c r="AN6" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="AO6">
+        <v>0.85915492957746398</v>
+      </c>
+      <c r="AP6">
+        <v>0.90140845070422504</v>
+      </c>
+      <c r="AQ6" s="15" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="15">
         <v>3</v>
       </c>
-      <c r="D7" s="17">
+      <c r="D7" s="16">
         <v>0.97299999999999998</v>
       </c>
-      <c r="E7" s="16">
+      <c r="E7" s="15">
         <v>1.4290000000000001E-2</v>
       </c>
-      <c r="H7" s="15">
-        <v>1</v>
-      </c>
-      <c r="I7" s="16">
-        <v>1</v>
-      </c>
-      <c r="J7" s="25">
-        <v>1</v>
-      </c>
-      <c r="K7" s="26">
-        <v>1</v>
-      </c>
-      <c r="L7" s="25">
-        <v>1</v>
-      </c>
-      <c r="M7" s="26">
-        <v>1</v>
-      </c>
-      <c r="N7" s="25">
-        <v>1</v>
-      </c>
-      <c r="O7" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A8" s="15" t="s">
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7" s="15">
+        <v>1</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+      <c r="K7" s="15">
+        <v>1</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7" s="15">
+        <v>1</v>
+      </c>
+      <c r="N7">
+        <v>1</v>
+      </c>
+      <c r="O7" s="15">
+        <v>1</v>
+      </c>
+      <c r="AC7">
+        <v>1</v>
+      </c>
+      <c r="AD7">
+        <v>0.81659999999999999</v>
+      </c>
+      <c r="AF7">
+        <v>0.36666666666666597</v>
+      </c>
+      <c r="AG7">
+        <v>0.36666666666666597</v>
+      </c>
+      <c r="AH7" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="AI7">
+        <v>0.36666666666666597</v>
+      </c>
+      <c r="AJ7">
+        <v>0.36666666666666597</v>
+      </c>
+      <c r="AK7" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL7">
+        <v>1</v>
+      </c>
+      <c r="AM7">
+        <v>1</v>
+      </c>
+      <c r="AN7" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO7">
+        <v>1</v>
+      </c>
+      <c r="AP7">
+        <v>0.63333333333333297</v>
+      </c>
+      <c r="AQ7" s="15" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="16">
+      <c r="C8" s="15">
         <v>2</v>
       </c>
-      <c r="D8" s="17">
+      <c r="D8" s="16">
         <v>0.71799999999999997</v>
       </c>
-      <c r="E8" s="16">
+      <c r="E8" s="15">
         <v>9.9299999999999996E-3</v>
       </c>
-      <c r="H8" s="15">
+      <c r="H8">
         <v>0.74350000000000005</v>
       </c>
-      <c r="I8" s="16">
+      <c r="I8" s="15">
         <v>0.74350000000000005</v>
       </c>
-      <c r="J8" s="25">
+      <c r="J8">
         <v>0.76060000000000005</v>
       </c>
-      <c r="K8" s="26">
+      <c r="K8" s="15">
         <v>0.76919999999999999</v>
       </c>
-      <c r="L8" s="25">
+      <c r="L8">
         <v>0.76919999999999999</v>
       </c>
-      <c r="M8" s="26">
+      <c r="M8" s="15">
         <v>0.75209999999999999</v>
       </c>
-      <c r="N8" s="25">
+      <c r="N8">
         <v>0.76919999999999999</v>
       </c>
-      <c r="O8" s="16">
+      <c r="O8" s="15">
         <v>0.79479999999999995</v>
       </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A9" s="15" t="s">
+      <c r="AC8">
+        <v>0.72219999999999995</v>
+      </c>
+      <c r="AD8">
+        <v>0.73070000000000002</v>
+      </c>
+      <c r="AF8">
+        <v>0.74358974358974295</v>
+      </c>
+      <c r="AG8">
+        <v>0.74358974358974295</v>
+      </c>
+      <c r="AH8" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="AI8">
+        <v>0.74358974358974295</v>
+      </c>
+      <c r="AJ8">
+        <v>0.74358974358974295</v>
+      </c>
+      <c r="AK8" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="AL8">
+        <v>0.67521367521367504</v>
+      </c>
+      <c r="AM8">
+        <v>0.60683760683760601</v>
+      </c>
+      <c r="AN8" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO8">
+        <v>0.74358974358974295</v>
+      </c>
+      <c r="AP8">
+        <v>0.72649572649572602</v>
+      </c>
+      <c r="AQ8" s="15" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B9" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="16">
+      <c r="C9" s="15">
         <v>2</v>
       </c>
-      <c r="D9" s="17">
+      <c r="D9" s="16">
         <v>0.77</v>
       </c>
-      <c r="E9" s="16">
+      <c r="E9" s="15">
         <v>1.4499999999999999E-3</v>
       </c>
-      <c r="H9" s="15">
+      <c r="H9">
         <v>0.78569999999999995</v>
       </c>
-      <c r="I9" s="16">
+      <c r="I9" s="15">
         <v>0.78569999999999995</v>
       </c>
-      <c r="J9" s="25">
+      <c r="J9">
         <v>0.73370000000000002</v>
       </c>
-      <c r="K9" s="26">
+      <c r="K9" s="15">
         <v>0.72719999999999996</v>
       </c>
-      <c r="L9" s="25">
+      <c r="L9">
         <v>0.74019999999999997</v>
       </c>
-      <c r="M9" s="26">
+      <c r="M9" s="15">
         <v>0.74670000000000003</v>
       </c>
-      <c r="N9" s="25">
+      <c r="N9">
         <v>0.75319999999999998</v>
       </c>
-      <c r="O9" s="26">
+      <c r="O9" s="15">
         <v>0.75319999999999998</v>
       </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A10" s="15" t="s">
+      <c r="AC9">
+        <v>0.75</v>
+      </c>
+      <c r="AD9">
+        <v>0.72719999999999996</v>
+      </c>
+      <c r="AF9">
+        <v>0.72077922077921996</v>
+      </c>
+      <c r="AG9">
+        <v>0.64285714285714202</v>
+      </c>
+      <c r="AH9" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI9">
+        <v>0.73376623376623296</v>
+      </c>
+      <c r="AJ9">
+        <v>0.75324675324675305</v>
+      </c>
+      <c r="AK9" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="AL9">
+        <v>0.75974025974025905</v>
+      </c>
+      <c r="AM9">
+        <v>0.76623376623376604</v>
+      </c>
+      <c r="AN9" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="AO9">
+        <v>0.70779220779220697</v>
+      </c>
+      <c r="AP9">
+        <v>0.71428571428571397</v>
+      </c>
+      <c r="AQ9" s="15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="15" t="s">
+      <c r="B10" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="16">
+      <c r="C10" s="15">
         <v>2</v>
       </c>
-      <c r="D10" s="17">
+      <c r="D10" s="16">
         <v>0.83199999999999996</v>
       </c>
-      <c r="E10" s="16">
+      <c r="E10" s="15">
         <v>5.4299999999999999E-3</v>
       </c>
-      <c r="H10" s="15">
+      <c r="H10">
         <v>0.88090000000000002</v>
       </c>
-      <c r="I10" s="16">
+      <c r="I10" s="15">
         <v>0.90469999999999995</v>
       </c>
-      <c r="J10" s="25">
+      <c r="J10">
         <v>0.90469999999999995</v>
       </c>
-      <c r="K10" s="26">
+      <c r="K10" s="15">
         <v>0.85709999999999997</v>
       </c>
-      <c r="L10" s="25">
+      <c r="L10">
         <v>0.92849999999999999</v>
       </c>
-      <c r="M10" s="26">
+      <c r="M10" s="15">
         <v>0.90469999999999995</v>
       </c>
-      <c r="N10" s="25">
+      <c r="N10">
         <v>0.92849999999999999</v>
       </c>
-      <c r="O10" s="26">
+      <c r="O10" s="15">
         <v>0.90469999999999995</v>
       </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A11" s="15" t="s">
+      <c r="AC10">
+        <v>0.83330000000000004</v>
+      </c>
+      <c r="AD10">
+        <v>0.84519999999999995</v>
+      </c>
+      <c r="AF10">
+        <v>0.66666666666666596</v>
+      </c>
+      <c r="AG10">
+        <v>0.59523809523809501</v>
+      </c>
+      <c r="AH10" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="AI10">
+        <v>0.66666666666666596</v>
+      </c>
+      <c r="AJ10">
+        <v>0.5</v>
+      </c>
+      <c r="AK10" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="AL10">
+        <v>0.76190476190476097</v>
+      </c>
+      <c r="AM10">
+        <v>0.66666666666666596</v>
+      </c>
+      <c r="AN10" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="AO10">
+        <v>0.88095238095238004</v>
+      </c>
+      <c r="AP10">
+        <v>0.61904761904761896</v>
+      </c>
+      <c r="AQ10" s="15" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B11" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="16">
+      <c r="C11" s="15">
         <v>3</v>
       </c>
-      <c r="D11" s="17">
+      <c r="D11" s="16">
         <v>0.99199999999999999</v>
       </c>
-      <c r="E11" s="16">
+      <c r="E11" s="15">
         <v>2.2599999999999999E-3</v>
       </c>
-      <c r="H11" s="15">
-        <v>1</v>
-      </c>
-      <c r="I11" s="16">
-        <v>1</v>
-      </c>
-      <c r="J11" s="25">
-        <v>1</v>
-      </c>
-      <c r="K11" s="26">
-        <v>1</v>
-      </c>
-      <c r="L11" s="25">
-        <v>1</v>
-      </c>
-      <c r="M11" s="26">
-        <v>1</v>
-      </c>
-      <c r="N11" s="25">
-        <v>1</v>
-      </c>
-      <c r="O11" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A12" s="25" t="s">
+      <c r="H11">
+        <v>1</v>
+      </c>
+      <c r="I11" s="15">
+        <v>1</v>
+      </c>
+      <c r="J11">
+        <v>1</v>
+      </c>
+      <c r="K11" s="15">
+        <v>1</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11" s="15">
+        <v>1</v>
+      </c>
+      <c r="N11">
+        <v>1</v>
+      </c>
+      <c r="O11" s="15">
+        <v>1</v>
+      </c>
+      <c r="AC11">
+        <v>0.98609999999999998</v>
+      </c>
+      <c r="AD11">
+        <v>0.93049999999999999</v>
+      </c>
+      <c r="AF11">
+        <v>0.47222222222222199</v>
+      </c>
+      <c r="AG11">
+        <v>0.61111111111111105</v>
+      </c>
+      <c r="AH11" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="AI11">
+        <v>0.55555555555555503</v>
+      </c>
+      <c r="AJ11">
+        <v>0.52777777777777701</v>
+      </c>
+      <c r="AK11" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL11">
+        <v>1</v>
+      </c>
+      <c r="AM11">
+        <v>1</v>
+      </c>
+      <c r="AN11" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="AO11">
+        <v>0.97222222222222199</v>
+      </c>
+      <c r="AP11">
+        <v>0.94444444444444398</v>
+      </c>
+      <c r="AQ11" s="15" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="25" t="s">
+      <c r="B12" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="16">
+      <c r="C12" s="15">
         <v>2</v>
       </c>
-      <c r="J12" s="25">
+      <c r="J12">
         <v>0.81640000000000001</v>
       </c>
-      <c r="K12" s="16">
+      <c r="K12" s="15">
         <v>0.82140000000000002</v>
       </c>
-      <c r="N12" s="25">
+      <c r="N12">
         <v>0.81689999999999996</v>
       </c>
-      <c r="O12" s="16">
+      <c r="O12" s="15">
         <v>0.82379999999999998</v>
       </c>
-      <c r="P12" s="28">
+      <c r="P12" s="23">
         <v>0.87129999999999996</v>
+      </c>
+      <c r="Q12">
+        <v>0.81953117002763798</v>
+      </c>
+      <c r="R12">
+        <v>0.81901934691370604</v>
+      </c>
+      <c r="S12" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="T12">
+        <v>0.818712253045347</v>
+      </c>
+      <c r="U12">
+        <v>0.81912171153649205</v>
+      </c>
+      <c r="V12" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="W12">
+        <v>0.81942880500000004</v>
+      </c>
+      <c r="X12">
+        <v>0.81840515899999999</v>
+      </c>
+      <c r="Y12" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z12">
+        <v>0.82598014126317898</v>
+      </c>
+      <c r="AA12">
+        <v>0.82669669362268405</v>
+      </c>
+      <c r="AB12" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="AC12">
+        <v>0.82640000000000002</v>
+      </c>
+      <c r="AD12">
+        <v>0.82530000000000003</v>
+      </c>
+      <c r="AF12">
+        <v>0.82003999999999999</v>
+      </c>
+      <c r="AG12">
+        <v>0.82330999999999999</v>
+      </c>
+      <c r="AI12">
+        <v>0.819735899273211</v>
+      </c>
+      <c r="AJ12">
+        <v>0.82157846248336497</v>
+      </c>
+      <c r="AK12" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="AL12">
+        <v>0.82567304739481995</v>
+      </c>
+      <c r="AM12">
+        <v>0.84512232572422896</v>
+      </c>
+      <c r="AN12" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="AO12">
+        <v>0.81748387757191099</v>
+      </c>
+      <c r="AP12">
+        <v>0.82024772238714305</v>
+      </c>
+      <c r="AQ12" s="15" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>78</v>
+      </c>
+      <c r="AL13">
+        <v>0.79066666699999999</v>
+      </c>
+      <c r="AM13">
+        <v>0.80033333299999998</v>
+      </c>
+      <c r="AN13" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="14" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>80</v>
+      </c>
+      <c r="AL14">
+        <v>0.89052305700000001</v>
+      </c>
+      <c r="AM14">
+        <v>0.84662169600000003</v>
+      </c>
+      <c r="AN14" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>